<commit_message>
Update model to v2 (GridSearchCV), fix class imbalance, and add audit documentation
</commit_message>
<xml_diff>
--- a/data/raw/event1_raw.xlsx
+++ b/data/raw/event1_raw.xlsx
@@ -6339,11 +6339,11 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Hotma Simanjuntak</t>
+          <t>Mardiana</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D104" t="inlineStr">
         <is>
@@ -6352,17 +6352,17 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Jl. Kalisari No. 36, RT.012/RW.002</t>
+          <t>Jl. Kayu Manis Barat No. 15 RT 019/004 Kayu Manis</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>Kalisari</t>
+          <t>Kayu Manis</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>Pasar Rebo</t>
+          <t>Matraman</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
@@ -6377,12 +6377,12 @@
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>9.3 KM</t>
+          <t>12 KM</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
         <is>
-          <t>Tidak Terdaftar</t>
+          <t>Terdaftar</t>
         </is>
       </c>
       <c r="L104" t="inlineStr">
@@ -6397,11 +6397,11 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Ayu Rahmawati</t>
+          <t>Aisyah Putri</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>43</v>
+        <v>66</v>
       </c>
       <c r="D105" t="inlineStr">
         <is>
@@ -6410,32 +6410,32 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Jl. Kalisari No. 130 RT 10 RW 01</t>
+          <t>Jl. Raya Bekasi Timur No. 33 RT 004/005 Bekasi Jaya</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>Utan Kayu Selatan</t>
+          <t>Bekasi Jaya</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>Matraman</t>
+          <t>Bekasi Timur</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>Jakarta Timur</t>
+          <t>Bekasi</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>DKI Jakarta</t>
+          <t>Jawa Barat</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>7.4 KM</t>
+          <t>16 KM</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
@@ -6445,7 +6445,7 @@
       </c>
       <c r="L105" t="inlineStr">
         <is>
-          <t>Hadir</t>
+          <t>Tidak Hadir</t>
         </is>
       </c>
     </row>
@@ -6455,11 +6455,11 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Fauziah Nurhayati</t>
+          <t>Supiah</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="D106" t="inlineStr">
         <is>
@@ -6468,22 +6468,22 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Jl. Tanjung Barat No. 72 RT 13 RW 01</t>
+          <t>Jl. Raya Bogor No. 88 RT 004/006 Ciracas</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>Pancoran</t>
+          <t>Ciracas</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>Pancoran</t>
+          <t>Ciracas</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>Jakarta Selatan</t>
+          <t>Jakarta Timur</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -6493,7 +6493,7 @@
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>6.0 KM</t>
+          <t>4.5 KM</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
@@ -6513,11 +6513,11 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Tuti Alawiyah</t>
+          <t>Nuraini</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="D107" t="inlineStr">
         <is>
@@ -6526,22 +6526,22 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Jl. Fatmawati No. 87 RT.2/RW.2</t>
+          <t>Jl. Garuda VII Pulo Gebang Permai No. 5 RT 002/003</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>Kalibata</t>
+          <t>Pulo Gebang</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>Pancoran</t>
+          <t>Cakung</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>Jakarta Selatan</t>
+          <t>Jakarta Timur</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -6551,12 +6551,12 @@
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>6.5 KM</t>
+          <t>11 KM</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
         <is>
-          <t>Terdaftar</t>
+          <t>Tidak Terdaftar</t>
         </is>
       </c>
       <c r="L107" t="inlineStr">
@@ -6571,45 +6571,45 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Rotua Simanullang</t>
+          <t>Agus Salim</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Perempuan</t>
+          <t>Laki - Laki</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Jl. Dewi Sartika No. 118 RT.9/RW.2</t>
+          <t>Jl. Raya Bekasi Timur No. 33 RT 004/005 Bekasi Jaya</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>Halim Perdanakusuma</t>
+          <t>Bekasi Jaya</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>Makasar</t>
+          <t>Bekasi Timur</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>Jakarta Timur</t>
+          <t>Bekasi</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>DKI Jakarta</t>
+          <t>Jawa Barat</t>
         </is>
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>1.9 KM</t>
+          <t>16 KM</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
@@ -6619,7 +6619,7 @@
       </c>
       <c r="L108" t="inlineStr">
         <is>
-          <t>Hadir</t>
+          <t>Tidak Hadir</t>
         </is>
       </c>
     </row>
@@ -6629,11 +6629,11 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Mardiyah</t>
+          <t>Umi Salamah</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>42</v>
+        <v>29</v>
       </c>
       <c r="D109" t="inlineStr">
         <is>
@@ -6642,22 +6642,22 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Jl. Pemuda No. 148, RT.004/RW.012</t>
+          <t>Jl. Sunter Mas Raya No. 18 RT 003/002 Sunter Jaya</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>Makasar</t>
+          <t>Sunter Jaya</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>Makasar</t>
+          <t>Tanjung Priok</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>Jakarta Timur</t>
+          <t>Jakarta Utara</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
@@ -6667,7 +6667,7 @@
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>870 M</t>
+          <t>19 KM</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
@@ -6677,7 +6677,7 @@
       </c>
       <c r="L109" t="inlineStr">
         <is>
-          <t>Hadir</t>
+          <t>Tidak Hadir</t>
         </is>
       </c>
     </row>
@@ -6687,11 +6687,11 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Khodijah</t>
+          <t>Nurjanah</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="D110" t="inlineStr">
         <is>
@@ -6700,22 +6700,22 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Jl. Raya Kramat Jati No. 60 RT.14/RW.2</t>
+          <t>Jl. Ciledug Raya No. 78 RT 002/004 Kebayoran Lama</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>Kebon Pala</t>
+          <t>Kebayoran Lama Utara</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>Makasar</t>
+          <t>Kebayoran Lama</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>Jakarta Timur</t>
+          <t>Jakarta Selatan</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -6725,7 +6725,7 @@
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>290 M</t>
+          <t>18 KM</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
@@ -6735,7 +6735,7 @@
       </c>
       <c r="L110" t="inlineStr">
         <is>
-          <t>Hadir</t>
+          <t>Tidak Hadir</t>
         </is>
       </c>
     </row>
@@ -6745,11 +6745,11 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Duma Simbolon</t>
+          <t>Sunarti</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="D111" t="inlineStr">
         <is>
@@ -6758,32 +6758,32 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Jl. Raya Pemuda No. 91, RT 04/RW 11</t>
+          <t>Jl. Margonda Raya No. 150 RT 005/003 Beji Depok</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>Kramat Jati</t>
+          <t>Beji</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>Kramat Jati</t>
+          <t>Beji</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>Jakarta Timur</t>
+          <t>Depok</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>DKI Jakarta</t>
+          <t>Jawa Barat</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>2.7 KM</t>
+          <t>22 KM</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
@@ -6793,7 +6793,7 @@
       </c>
       <c r="L111" t="inlineStr">
         <is>
-          <t>Hadir</t>
+          <t>Tidak Hadir</t>
         </is>
       </c>
     </row>
@@ -6803,11 +6803,11 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Fatimah Zahra</t>
+          <t>Fatmawati</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>40</v>
+        <v>64</v>
       </c>
       <c r="D112" t="inlineStr">
         <is>
@@ -6816,22 +6816,22 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Jl. Raya Pasar Minggu No. 44 RT 09 RW 12</t>
+          <t>Jl. Muara Baru No. 9 RT 007/001 Penjaringan Jakut</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>Duren Tiga</t>
+          <t>Penjaringan</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>Pancoran</t>
+          <t>Penjaringan</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>Jakarta Selatan</t>
+          <t>Jakarta Utara</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
@@ -6841,12 +6841,12 @@
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>6.8 KM</t>
+          <t>26 KM</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
         <is>
-          <t>Tidak Terdaftar</t>
+          <t>Terdaftar</t>
         </is>
       </c>
       <c r="L112" t="inlineStr">
@@ -6861,11 +6861,11 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Saroh</t>
+          <t>Maisyaroh</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>49</v>
+        <v>65</v>
       </c>
       <c r="D113" t="inlineStr">
         <is>
@@ -6874,22 +6874,22 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Jl. Kalisari No. 84 RT 14 RW 01</t>
+          <t>Jl. Yos Sudarso No. 55 RT 009/001 Sukapura Cilincing</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>Cipinang Melayu</t>
+          <t>Sukapura</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>Makasar</t>
+          <t>Cilincing</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>Jakarta Timur</t>
+          <t>Jakarta Utara</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -6899,7 +6899,7 @@
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>1.7 KM</t>
+          <t>24 KM</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
@@ -6909,7 +6909,7 @@
       </c>
       <c r="L113" t="inlineStr">
         <is>
-          <t>Hadir</t>
+          <t>Tidak Hadir</t>
         </is>
       </c>
     </row>
@@ -6919,11 +6919,11 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Rukmini</t>
+          <t>Murniati</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="D114" t="inlineStr">
         <is>
@@ -6932,17 +6932,17 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Jl. Raya Ahmad Yani No. 55, RT 15/RW 10</t>
+          <t>Jl. Jatiwaringin Raya No. 45 RT 006/003 Jatiwaringin</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>Bintara</t>
+          <t>Jatiwaringin</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>Bekasi Barat</t>
+          <t>Pondok Gede</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
@@ -6957,7 +6957,7 @@
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>11.2 KM</t>
+          <t>11 KM</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
@@ -6977,11 +6977,11 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Lestari Nababan</t>
+          <t>Komariah</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>40</v>
+        <v>56</v>
       </c>
       <c r="D115" t="inlineStr">
         <is>
@@ -6990,32 +6990,32 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Jl. Batu Ampar No. 37 RT 05 RW 03</t>
+          <t>Jl. Transyogi Cibubur No. 8 RT 007/002 Cibubur</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>Cililitan</t>
+          <t>Cibubur</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>Kramat Jati</t>
+          <t>Cibubur</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>Jakarta Timur</t>
+          <t>Kota Bekasi</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>DKI Jakarta</t>
+          <t>Jawa Barat</t>
         </is>
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>1.6 KM</t>
+          <t>13 KM</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -7035,11 +7035,11 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Suminah</t>
+          <t>Hayati</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>46</v>
+        <v>65</v>
       </c>
       <c r="D116" t="inlineStr">
         <is>
@@ -7048,22 +7048,22 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Jl. Lenteng Agung No. 150 RT 07 RW 06</t>
+          <t>Jl. Muara Baru No. 9 RT 007/001 Penjaringan Jakut</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>Lenteng Agung</t>
+          <t>Penjaringan</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>Jagakarsa</t>
+          <t>Penjaringan</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>Jakarta Selatan</t>
+          <t>Jakarta Utara</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -7073,7 +7073,7 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>11.3 KM</t>
+          <t>26 KM</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -7083,7 +7083,7 @@
       </c>
       <c r="L116" t="inlineStr">
         <is>
-          <t>Hadir</t>
+          <t>Tidak Hadir</t>
         </is>
       </c>
     </row>
@@ -7093,45 +7093,45 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Fenny Marliana</t>
+          <t>Wahyu Santoso</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>27</v>
+        <v>56</v>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Perempuan</t>
+          <t>Laki - Laki</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Jl. Cilincing Raya No. 29 RT 03 RW 11</t>
+          <t>Jl. Dewi Sartika No. 4 RT 001/002 Ciputat Tangsel</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>Cilincing</t>
+          <t>Ciputat</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>Cilincing</t>
+          <t>Ciputat</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>Jakarta Utara</t>
+          <t>Tangerang Selatan</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>DKI Jakarta</t>
+          <t>Banten</t>
         </is>
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>16.7 KM</t>
+          <t>30 KM</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -7141,7 +7141,7 @@
       </c>
       <c r="L117" t="inlineStr">
         <is>
-          <t>Hadir</t>
+          <t>Tidak Hadir</t>
         </is>
       </c>
     </row>
@@ -7151,11 +7151,11 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Iis Solihat</t>
+          <t>Eka Fitriani</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>29</v>
+        <v>50</v>
       </c>
       <c r="D118" t="inlineStr">
         <is>
@@ -7164,22 +7164,22 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Jl. Lenteng Agung No. 120, RT.009/RW.005</t>
+          <t>Jl. Garuda VII Pulo Gebang Permai No. 5 RT 002/003</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>Pasar Manggis</t>
+          <t>Pulo Gebang</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>Setiabudi</t>
+          <t>Cakung</t>
         </is>
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>Jakarta Selatan</t>
+          <t>Jakarta Timur</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -7189,7 +7189,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>9.1 KM</t>
+          <t>11 KM</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -7199,7 +7199,7 @@
       </c>
       <c r="L118" t="inlineStr">
         <is>
-          <t>Hadir</t>
+          <t>Tidak Hadir</t>
         </is>
       </c>
     </row>
@@ -7209,11 +7209,11 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Bella Permata</t>
+          <t>Aminah</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>39</v>
+        <v>51</v>
       </c>
       <c r="D119" t="inlineStr">
         <is>
@@ -7222,22 +7222,22 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Jl. Raya Fatmawati No. 69, RT 13/RW 11</t>
+          <t>Jl. Muara Baru No. 9 RT 007/001 Penjaringan Jakut</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>Tebet Barat</t>
+          <t>Penjaringan</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>Tebet</t>
+          <t>Penjaringan</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>Jakarta Selatan</t>
+          <t>Jakarta Utara</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -7247,7 +7247,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>4.0 KM</t>
+          <t>26 KM</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -7257,7 +7257,7 @@
       </c>
       <c r="L119" t="inlineStr">
         <is>
-          <t>Hadir</t>
+          <t>Tidak Hadir</t>
         </is>
       </c>
     </row>
@@ -7267,11 +7267,11 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Meyla Septiana</t>
+          <t>Supriyati</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="D120" t="inlineStr">
         <is>
@@ -7280,32 +7280,32 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Jl. Bekasi Raya No. 129, RT.013/RW.003</t>
+          <t>Jl. Margonda Raya No. 150 RT 005/003 Beji Depok</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>Halim Perdanakusuma</t>
+          <t>Beji</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>Makasar</t>
+          <t>Beji</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>Jakarta Timur</t>
+          <t>Depok</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>DKI Jakarta</t>
+          <t>Jawa Barat</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>840 M</t>
+          <t>22 KM</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -7315,7 +7315,7 @@
       </c>
       <c r="L120" t="inlineStr">
         <is>
-          <t>Hadir</t>
+          <t>Tidak Hadir</t>
         </is>
       </c>
     </row>
@@ -7325,11 +7325,11 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Dwi Rahmawati</t>
+          <t>Hindun</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D121" t="inlineStr">
         <is>
@@ -7338,32 +7338,32 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Jl. Margahayu Raya No. 51 RT 03 RW 06</t>
+          <t>Jl. Dewi Sartika No. 8 RT 003/005 Cililitan</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>Jatiwaringin</t>
+          <t>Cililitan</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>Pondok Gede</t>
+          <t>Kramat Jati</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>Bekasi</t>
+          <t>Jakarta Timur</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>Jawa Barat</t>
+          <t>DKI Jakarta</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>9.7 KM</t>
+          <t>2 KM</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -7373,7 +7373,7 @@
       </c>
       <c r="L121" t="inlineStr">
         <is>
-          <t>Tidak Hadir</t>
+          <t>Hadir</t>
         </is>
       </c>
     </row>
@@ -7383,11 +7383,11 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Tri Wahyuningsih</t>
+          <t>Wulandari</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>36</v>
+        <v>63</v>
       </c>
       <c r="D122" t="inlineStr">
         <is>
@@ -7396,32 +7396,32 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Jl. Raya Makasar No. 83, RT.008/RW.001</t>
+          <t>Jl. Boulevard Serpong No. 21 RT 003/001 Serpong</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>Kampung Melayu</t>
+          <t>Serpong</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>Jatinegara</t>
+          <t>Serpong</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>Jakarta Timur</t>
+          <t>Tangerang Selatan</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>DKI Jakarta</t>
+          <t>Banten</t>
         </is>
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>6.5 KM</t>
+          <t>35 KM</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -7441,11 +7441,11 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Yuliani</t>
+          <t>Dewi Lestari</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>31</v>
+        <v>63</v>
       </c>
       <c r="D123" t="inlineStr">
         <is>
@@ -7454,32 +7454,32 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Jl. Raya Kukusan No. 62, RT.001/RW.004</t>
+          <t>Jl. Garuda VII Pulo Gebang Permai No. 5 RT 002/003</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>Mekarsari</t>
+          <t>Pulo Gebang</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>Cimanggis</t>
+          <t>Cakung</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>Depok</t>
+          <t>Jakarta Timur</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>Jawa Barat</t>
+          <t>DKI Jakarta</t>
         </is>
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>11.7 KM</t>
+          <t>11 KM</t>
         </is>
       </c>
       <c r="K123" t="inlineStr">
@@ -7489,7 +7489,7 @@
       </c>
       <c r="L123" t="inlineStr">
         <is>
-          <t>Hadir</t>
+          <t>Tidak Hadir</t>
         </is>
       </c>
     </row>
@@ -7499,11 +7499,11 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Sri Wahyuni</t>
+          <t>Endang Susanti</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>57</v>
+        <v>34</v>
       </c>
       <c r="D124" t="inlineStr">
         <is>
@@ -7512,17 +7512,17 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Jl. Penggilingan No. 33 RT 11 RW 08</t>
+          <t>Jl. Dewi Sartika No. 8 RT 003/005 Cililitan</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>Makasar</t>
+          <t>Cililitan</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>Makasar</t>
+          <t>Kramat Jati</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
@@ -7537,17 +7537,17 @@
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>1.1 KM</t>
+          <t>2 KM</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
         <is>
-          <t>Tidak Terdaftar</t>
+          <t>Terdaftar</t>
         </is>
       </c>
       <c r="L124" t="inlineStr">
         <is>
-          <t>Tidak Hadir</t>
+          <t>Hadir</t>
         </is>
       </c>
     </row>
@@ -7557,11 +7557,11 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Kasmini</t>
+          <t>Nurhayati</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="D125" t="inlineStr">
         <is>
@@ -7570,22 +7570,22 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Jl. Pasar Rebo No. 139 RT 13 RW 12</t>
+          <t>Jl. Sunter Mas Raya No. 18 RT 003/002 Sunter Jaya</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>Cililitan</t>
+          <t>Sunter Jaya</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>Kramat Jati</t>
+          <t>Tanjung Priok</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>Jakarta Timur</t>
+          <t>Jakarta Utara</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
@@ -7595,7 +7595,7 @@
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>2.5 KM</t>
+          <t>19 KM</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
@@ -7615,11 +7615,11 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Sukarsih</t>
+          <t>Erni Rahayu</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="D126" t="inlineStr">
         <is>
@@ -7628,22 +7628,22 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Jl. Duren Tiga No. 113 RT.15/RW.9</t>
+          <t>Jl. Muara Baru No. 9 RT 007/001 Penjaringan Jakut</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>Kalibata</t>
+          <t>Penjaringan</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>Pancoran</t>
+          <t>Penjaringan</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>Jakarta Selatan</t>
+          <t>Jakarta Utara</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -7653,7 +7653,7 @@
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>5.3 KM</t>
+          <t>26 KM</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
@@ -7663,7 +7663,7 @@
       </c>
       <c r="L126" t="inlineStr">
         <is>
-          <t>Hadir</t>
+          <t>Tidak Hadir</t>
         </is>
       </c>
     </row>
@@ -7673,11 +7673,11 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Haryanti</t>
+          <t>Wati Susanti</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>31</v>
+        <v>47</v>
       </c>
       <c r="D127" t="inlineStr">
         <is>
@@ -7686,7 +7686,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Jl. Kalisari No. 57, RT.001/RW.002</t>
+          <t>Jl. Kamboja No. 12 RT 002/001 Kebon Pala</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
@@ -7711,17 +7711,17 @@
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>280 M</t>
+          <t>600 M</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
         <is>
-          <t>Tidak Terdaftar</t>
+          <t>Terdaftar</t>
         </is>
       </c>
       <c r="L127" t="inlineStr">
         <is>
-          <t>Tidak Hadir</t>
+          <t>Hadir</t>
         </is>
       </c>
     </row>
@@ -7731,11 +7731,11 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Mulyani</t>
+          <t>Siti Rohani</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>39</v>
+        <v>62</v>
       </c>
       <c r="D128" t="inlineStr">
         <is>
@@ -7744,32 +7744,32 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Jl. Kalimalang No. 132 RT.4/RW.5</t>
+          <t>Jl. Jatiwaringin Raya No. 45 RT 006/003 Jatiwaringin</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>Cawang</t>
+          <t>Jatiwaringin</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>Kramat Jati</t>
+          <t>Pondok Gede</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>Jakarta Timur</t>
+          <t>Bekasi</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>DKI Jakarta</t>
+          <t>Jawa Barat</t>
         </is>
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>1.5 KM</t>
+          <t>11 KM</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
@@ -7789,11 +7789,11 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Rukaiyah</t>
+          <t>Wahyuni</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>45</v>
+        <v>67</v>
       </c>
       <c r="D129" t="inlineStr">
         <is>
@@ -7802,32 +7802,32 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Jl. Damai No. 63 RT.13/RW.8</t>
+          <t>Jl. Margonda Raya No. 150 RT 005/003 Beji Depok</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>Balekambang</t>
+          <t>Beji</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>Kramat Jati</t>
+          <t>Beji</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>Jakarta Timur</t>
+          <t>Depok</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>DKI Jakarta</t>
+          <t>Jawa Barat</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>2.1 KM</t>
+          <t>22 KM</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
@@ -7837,7 +7837,7 @@
       </c>
       <c r="L129" t="inlineStr">
         <is>
-          <t>Hadir</t>
+          <t>Tidak Hadir</t>
         </is>
       </c>
     </row>
@@ -7847,11 +7847,11 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Fitriani</t>
+          <t>Srimulyani</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>34</v>
+        <v>64</v>
       </c>
       <c r="D130" t="inlineStr">
         <is>
@@ -7860,22 +7860,22 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Jl. Inpres No. 106, RT.008/RW.012</t>
+          <t>Jl. Muara Baru No. 9 RT 007/001 Penjaringan Jakut</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>Dukuh</t>
+          <t>Penjaringan</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>Kramat Jati</t>
+          <t>Penjaringan</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>Jakarta Timur</t>
+          <t>Jakarta Utara</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -7885,7 +7885,7 @@
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>3.0 KM</t>
+          <t>26 KM</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
@@ -7895,7 +7895,7 @@
       </c>
       <c r="L130" t="inlineStr">
         <is>
-          <t>Hadir</t>
+          <t>Tidak Hadir</t>
         </is>
       </c>
     </row>
@@ -7905,11 +7905,11 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Mujiati</t>
+          <t>Teti Haryati</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D131" t="inlineStr">
         <is>
@@ -7918,22 +7918,22 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Jl. Lenteng Agung No. 87 RT 13 RW 02</t>
+          <t>Jl. Kayu Manis Barat No. 15 RT 019/004 Kayu Manis</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>Kebon Baru</t>
+          <t>Kayu Manis</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>Tebet</t>
+          <t>Matraman</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>Jakarta Selatan</t>
+          <t>Jakarta Timur</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -7943,7 +7943,7 @@
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>6.7 KM</t>
+          <t>12 KM</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
@@ -7953,7 +7953,7 @@
       </c>
       <c r="L131" t="inlineStr">
         <is>
-          <t>Hadir</t>
+          <t>Tidak Hadir</t>
         </is>
       </c>
     </row>
@@ -7963,11 +7963,11 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Euis Kartini</t>
+          <t>Suryani</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="D132" t="inlineStr">
         <is>
@@ -7976,17 +7976,17 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Jl. Pondok Ranggon No. 72, RT.008/RW.004</t>
+          <t>Jl. Raya Bogor No. 88 RT 004/006 Ciracas</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>Dukuh</t>
+          <t>Ciracas</t>
         </is>
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>Kramat Jati</t>
+          <t>Ciracas</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
@@ -8001,12 +8001,12 @@
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>3.3 KM</t>
+          <t>4.5 KM</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>Terdaftar</t>
+          <t>Tidak Terdaftar</t>
         </is>
       </c>
       <c r="L132" t="inlineStr">
@@ -8021,11 +8021,11 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Sarmauli Siregar</t>
+          <t>Rubiyah</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="D133" t="inlineStr">
         <is>
@@ -8034,22 +8034,22 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Jl. Raya Bogor No. 139, RT.014/RW.001</t>
+          <t>Jl. Raya Ps. Minggu No. 99 RT 005/004 Pasar Minggu</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>Rambutan</t>
+          <t>Pasar Minggu</t>
         </is>
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>Ciracas</t>
+          <t>Pasar Minggu</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>Jakarta Timur</t>
+          <t>Jakarta Selatan</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
@@ -8059,7 +8059,7 @@
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>6.9 KM</t>
+          <t>14 KM</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
@@ -8069,7 +8069,7 @@
       </c>
       <c r="L133" t="inlineStr">
         <is>
-          <t>Hadir</t>
+          <t>Tidak Hadir</t>
         </is>
       </c>
     </row>
@@ -8079,45 +8079,45 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Eti Sumiati</t>
+          <t>Adi Prasetyo</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Perempuan</t>
+          <t>Laki - Laki</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Jl. Tanah Baru No. 124, RT.004/RW.007</t>
+          <t>Jl. Kramat Jati Raya No. 22 RT 007/004</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>Pasir Gunung Selatan</t>
+          <t>Kramat Jati</t>
         </is>
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>Cimanggis</t>
+          <t>Kramat Jati</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>Depok</t>
+          <t>Jakarta Timur</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>Jawa Barat</t>
+          <t>DKI Jakarta</t>
         </is>
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>11.3 KM</t>
+          <t>2.5 KM</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
@@ -8137,11 +8137,11 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Hesti Wulandari</t>
+          <t>Rosdiana</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D135" t="inlineStr">
         <is>
@@ -8150,32 +8150,32 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>Jl. Batu Ampar No. 74 RT.7/RW.12</t>
+          <t>Jl. Raya Bekasi Timur No. 33 RT 004/005 Bekasi Jaya</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>Halim Perdanakusuma</t>
+          <t>Bekasi Jaya</t>
         </is>
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>Makasar</t>
+          <t>Bekasi Timur</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>Jakarta Timur</t>
+          <t>Bekasi</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>DKI Jakarta</t>
+          <t>Jawa Barat</t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>320 M</t>
+          <t>16 KM</t>
         </is>
       </c>
       <c r="K135" t="inlineStr">
@@ -8185,7 +8185,7 @@
       </c>
       <c r="L135" t="inlineStr">
         <is>
-          <t>Hadir</t>
+          <t>Tidak Hadir</t>
         </is>
       </c>
     </row>
@@ -8195,11 +8195,11 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Nining Srimulyani</t>
+          <t>Sumiarsih</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="D136" t="inlineStr">
         <is>
@@ -8208,32 +8208,32 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>Jl. Raya Bogor No. 81 RT.1/RW.1</t>
+          <t>Jl. Dewi Sartika No. 4 RT 001/002 Ciputat Tangsel</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>Cipinang Besar Selatan</t>
+          <t>Ciputat</t>
         </is>
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>Makasar</t>
+          <t>Ciputat</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>Jakarta Timur</t>
+          <t>Tangerang Selatan</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>DKI Jakarta</t>
+          <t>Banten</t>
         </is>
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>1.6 KM</t>
+          <t>30 KM</t>
         </is>
       </c>
       <c r="K136" t="inlineStr">
@@ -8243,7 +8243,7 @@
       </c>
       <c r="L136" t="inlineStr">
         <is>
-          <t>Hadir</t>
+          <t>Tidak Hadir</t>
         </is>
       </c>
     </row>
@@ -8253,30 +8253,30 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Nunung Nurhayati</t>
+          <t>Eko Purnomo</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Perempuan</t>
+          <t>Laki - Laki</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>Jl. Cipinang Besar No. 21, RT.014/RW.003</t>
+          <t>Jl. Kayu Manis Barat No. 15 RT 019/004 Kayu Manis</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>Kayu Putih</t>
+          <t>Kayu Manis</t>
         </is>
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>Pulo Gadung</t>
+          <t>Matraman</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
@@ -8291,12 +8291,12 @@
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>7.9 KM</t>
+          <t>12 KM</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>Tidak Terdaftar</t>
+          <t>Terdaftar</t>
         </is>
       </c>
       <c r="L137" t="inlineStr">
@@ -8311,11 +8311,11 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Lisna Marlina</t>
+          <t>Titin Suprihatin</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="D138" t="inlineStr">
         <is>
@@ -8324,32 +8324,32 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Jl. Raya Condet No. 146, RT.004/RW.010</t>
+          <t>Jl. Dewi Sartika No. 4 RT 001/002 Ciputat Tangsel</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>Palmeriam</t>
+          <t>Ciputat</t>
         </is>
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>Matraman</t>
+          <t>Ciputat</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>Jakarta Timur</t>
+          <t>Tangerang Selatan</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>DKI Jakarta</t>
+          <t>Banten</t>
         </is>
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>8.5 KM</t>
+          <t>30 KM</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
@@ -8359,7 +8359,7 @@
       </c>
       <c r="L138" t="inlineStr">
         <is>
-          <t>Hadir</t>
+          <t>Tidak Hadir</t>
         </is>
       </c>
     </row>
@@ -8369,11 +8369,11 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Roida Siahaan</t>
+          <t>Septiani</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="D139" t="inlineStr">
         <is>
@@ -8382,17 +8382,17 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Jl. Raya Pengairan No. 81 RT 15 RW 05</t>
+          <t>Jl. Kayu Manis Barat No. 15 RT 019/004 Kayu Manis</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>Cijantung</t>
+          <t>Kayu Manis</t>
         </is>
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>Pasar Rebo</t>
+          <t>Matraman</t>
         </is>
       </c>
       <c r="H139" t="inlineStr">
@@ -8407,7 +8407,7 @@
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>8.2 KM</t>
+          <t>12 KM</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
@@ -8417,7 +8417,7 @@
       </c>
       <c r="L139" t="inlineStr">
         <is>
-          <t>Hadir</t>
+          <t>Tidak Hadir</t>
         </is>
       </c>
     </row>
@@ -8427,11 +8427,11 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Siti Aminah</t>
+          <t>Hartini</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="D140" t="inlineStr">
         <is>
@@ -8440,32 +8440,32 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>Jl. Kalibata Raya No. 77, RT.008/RW.006</t>
+          <t>Jl. Bintara Jaya No. 7 RT 003/002 Bintara Jaya Bekasi</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>Tebet Barat</t>
+          <t>Bintara Jaya</t>
         </is>
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>Tebet</t>
+          <t>Bekasi Barat</t>
         </is>
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>Jakarta Selatan</t>
+          <t>Bekasi</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>DKI Jakarta</t>
+          <t>Jawa Barat</t>
         </is>
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>5.5 KM</t>
+          <t>13 KM</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
@@ -8475,7 +8475,7 @@
       </c>
       <c r="L140" t="inlineStr">
         <is>
-          <t>Hadir</t>
+          <t>Tidak Hadir</t>
         </is>
       </c>
     </row>
@@ -8485,11 +8485,11 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Sari Nuraini</t>
+          <t>Pariyem</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>27</v>
+        <v>47</v>
       </c>
       <c r="D141" t="inlineStr">
         <is>
@@ -8498,32 +8498,32 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Jl. Raya Inspeksi Kalimalang No. 19, RT 09/RW 04</t>
+          <t>Jl. Bintara Jaya No. 7 RT 003/002 Bintara Jaya Bekasi</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>Cipinang Besar Selatan</t>
+          <t>Bintara Jaya</t>
         </is>
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>Makasar</t>
+          <t>Bekasi Barat</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>Jakarta Timur</t>
+          <t>Bekasi</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>DKI Jakarta</t>
+          <t>Jawa Barat</t>
         </is>
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>1.4 KM</t>
+          <t>13 KM</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
@@ -8533,7 +8533,7 @@
       </c>
       <c r="L141" t="inlineStr">
         <is>
-          <t>Hadir</t>
+          <t>Tidak Hadir</t>
         </is>
       </c>
     </row>
@@ -8543,11 +8543,11 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Lastri Utami</t>
+          <t>Salmah</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>32</v>
+        <v>53</v>
       </c>
       <c r="D142" t="inlineStr">
         <is>
@@ -8556,32 +8556,32 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>Jl. Pulo Gebang No. 95 RT.5/RW.3</t>
+          <t>Jl. Boulevard Serpong No. 21 RT 003/001 Serpong</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>Kebon Pala</t>
+          <t>Serpong</t>
         </is>
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>Makasar</t>
+          <t>Serpong</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>Jakarta Timur</t>
+          <t>Tangerang Selatan</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>DKI Jakarta</t>
+          <t>Banten</t>
         </is>
       </c>
       <c r="J142" t="inlineStr">
         <is>
-          <t>820 M</t>
+          <t>35 KM</t>
         </is>
       </c>
       <c r="K142" t="inlineStr">
@@ -8591,7 +8591,7 @@
       </c>
       <c r="L142" t="inlineStr">
         <is>
-          <t>Hadir</t>
+          <t>Tidak Hadir</t>
         </is>
       </c>
     </row>
@@ -8601,11 +8601,11 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Indah Permata Sari</t>
+          <t>Novia Anggraeni</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="D143" t="inlineStr">
         <is>
@@ -8614,32 +8614,32 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>Jl. Raya Kranggan No. 136, RT 01/RW 11</t>
+          <t>Jl. Garuda VII Pulo Gebang Permai No. 5 RT 002/003</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>Jaka Sampurna</t>
+          <t>Pulo Gebang</t>
         </is>
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>Bekasi Barat</t>
+          <t>Cakung</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>Bekasi</t>
+          <t>Jakarta Timur</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>Jawa Barat</t>
+          <t>DKI Jakarta</t>
         </is>
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>11.6 KM</t>
+          <t>11 KM</t>
         </is>
       </c>
       <c r="K143" t="inlineStr">
@@ -8649,7 +8649,7 @@
       </c>
       <c r="L143" t="inlineStr">
         <is>
-          <t>Hadir</t>
+          <t>Tidak Hadir</t>
         </is>
       </c>
     </row>
@@ -8659,11 +8659,11 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>Septiana Dewi</t>
+          <t>Karmiati</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D144" t="inlineStr">
         <is>
@@ -8672,22 +8672,22 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>Jl. Raya Kukusan No. 30 RT 15 RW 02</t>
+          <t>Jl. Raya Bekasi Timur No. 33 RT 004/005 Bekasi Jaya</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>Pasir Gunung Selatan</t>
+          <t>Bekasi Jaya</t>
         </is>
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>Cimanggis</t>
+          <t>Bekasi Timur</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>Depok</t>
+          <t>Bekasi</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
@@ -8697,7 +8697,7 @@
       </c>
       <c r="J144" t="inlineStr">
         <is>
-          <t>13.5 KM</t>
+          <t>16 KM</t>
         </is>
       </c>
       <c r="K144" t="inlineStr">
@@ -8707,7 +8707,7 @@
       </c>
       <c r="L144" t="inlineStr">
         <is>
-          <t>Hadir</t>
+          <t>Tidak Hadir</t>
         </is>
       </c>
     </row>
@@ -8717,11 +8717,11 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Yeni Rahmawati</t>
+          <t>Lela Wati</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="D145" t="inlineStr">
         <is>
@@ -8730,32 +8730,32 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>Jl. Raya Pasar Rebo No. 68, RT 09/RW 08</t>
+          <t>Jl. Raya Bogor KM 37 No. 12 RT 004/001 Curug</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>Balekambang</t>
+          <t>Curug</t>
         </is>
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>Kramat Jati</t>
+          <t>Cimanggis</t>
         </is>
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>Jakarta Timur</t>
+          <t>Depok</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>DKI Jakarta</t>
+          <t>Jawa Barat</t>
         </is>
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>1.9 KM</t>
+          <t>14 KM</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">
@@ -8765,7 +8765,7 @@
       </c>
       <c r="L145" t="inlineStr">
         <is>
-          <t>Hadir</t>
+          <t>Tidak Hadir</t>
         </is>
       </c>
     </row>
@@ -8775,11 +8775,11 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>Supriatin</t>
+          <t>Yayah Sumiyah</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D146" t="inlineStr">
         <is>
@@ -8788,32 +8788,32 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>Jl. Raya Raya Pondok Gede No. 71, RT 01/RW 01</t>
+          <t>Jl. Prof. Soepomo No. 27 RT 006/003 Tebet Barat</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>Jatiwaringin</t>
+          <t>Tebet Barat</t>
         </is>
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>Pondok Gede</t>
+          <t>Tebet</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>Bekasi</t>
+          <t>Jakarta Selatan</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>Jawa Barat</t>
+          <t>DKI Jakarta</t>
         </is>
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>8.0 KM</t>
+          <t>12 KM</t>
         </is>
       </c>
       <c r="K146" t="inlineStr">
@@ -8823,7 +8823,7 @@
       </c>
       <c r="L146" t="inlineStr">
         <is>
-          <t>Hadir</t>
+          <t>Tidak Hadir</t>
         </is>
       </c>
     </row>
@@ -8833,11 +8833,11 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Retno Dwi Astuti</t>
+          <t>Mariana Sari</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>41</v>
+        <v>61</v>
       </c>
       <c r="D147" t="inlineStr">
         <is>
@@ -8846,32 +8846,32 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>Jl. Cilandak No. 114 RT.9/RW.12</t>
+          <t>Jl. Raya Bogor KM 37 No. 12 RT 004/001 Curug</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>Pasar Manggis</t>
+          <t>Curug</t>
         </is>
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>Setiabudi</t>
+          <t>Cimanggis</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>Jakarta Selatan</t>
+          <t>Depok</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>DKI Jakarta</t>
+          <t>Jawa Barat</t>
         </is>
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>8.9 KM</t>
+          <t>14 KM</t>
         </is>
       </c>
       <c r="K147" t="inlineStr">
@@ -8881,7 +8881,7 @@
       </c>
       <c r="L147" t="inlineStr">
         <is>
-          <t>Hadir</t>
+          <t>Tidak Hadir</t>
         </is>
       </c>
     </row>
@@ -8891,11 +8891,11 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Yati Rosmiati</t>
+          <t>Cicih Suryani</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>31</v>
+        <v>59</v>
       </c>
       <c r="D148" t="inlineStr">
         <is>
@@ -8904,32 +8904,32 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>Jl. Raya Cipayung No. 140 RT 01 RW 06</t>
+          <t>Jl. Boulevard Serpong No. 21 RT 003/001 Serpong</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>Kampung Melayu</t>
+          <t>Serpong</t>
         </is>
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>Jatinegara</t>
+          <t>Serpong</t>
         </is>
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>Jakarta Timur</t>
+          <t>Tangerang Selatan</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
         <is>
-          <t>DKI Jakarta</t>
+          <t>Banten</t>
         </is>
       </c>
       <c r="J148" t="inlineStr">
         <is>
-          <t>4.6 KM</t>
+          <t>35 KM</t>
         </is>
       </c>
       <c r="K148" t="inlineStr">
@@ -8939,7 +8939,7 @@
       </c>
       <c r="L148" t="inlineStr">
         <is>
-          <t>Hadir</t>
+          <t>Tidak Hadir</t>
         </is>
       </c>
     </row>
@@ -8949,11 +8949,11 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Ningsih Saodah</t>
+          <t>Rini Handayani</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="D149" t="inlineStr">
         <is>
@@ -8962,17 +8962,17 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>Jl. Dewi Sartika No. 92 RT 04 RW 11</t>
+          <t>Jl. Kramat Jati Raya No. 22 RT 007/004</t>
         </is>
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>Cibubur</t>
+          <t>Kramat Jati</t>
         </is>
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>Ciracas</t>
+          <t>Kramat Jati</t>
         </is>
       </c>
       <c r="H149" t="inlineStr">
@@ -8987,7 +8987,7 @@
       </c>
       <c r="J149" t="inlineStr">
         <is>
-          <t>8.7 KM</t>
+          <t>2.5 KM</t>
         </is>
       </c>
       <c r="K149" t="inlineStr">
@@ -9007,11 +9007,11 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Fauzan Arifin</t>
+          <t>Budi Hartono</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="D150" t="inlineStr">
         <is>
@@ -9020,17 +9020,17 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>Jl. Radio Dalam No. 105 RT 10 RW 12</t>
+          <t>Jl. Raya Ps. Minggu No. 99 RT 005/004 Pasar Minggu</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>Menteng Dalam</t>
+          <t>Pasar Minggu</t>
         </is>
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>Tebet</t>
+          <t>Pasar Minggu</t>
         </is>
       </c>
       <c r="H150" t="inlineStr">
@@ -9045,7 +9045,7 @@
       </c>
       <c r="J150" t="inlineStr">
         <is>
-          <t>4.9 KM</t>
+          <t>14 KM</t>
         </is>
       </c>
       <c r="K150" t="inlineStr">
@@ -9055,7 +9055,7 @@
       </c>
       <c r="L150" t="inlineStr">
         <is>
-          <t>Hadir</t>
+          <t>Tidak Hadir</t>
         </is>
       </c>
     </row>
@@ -9065,11 +9065,11 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>Ahmad Fauzi</t>
+          <t>Hermanto</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="D151" t="inlineStr">
         <is>
@@ -9078,32 +9078,32 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>Jl. Raya Raya Tapos No. 106, RT 01/RW 03</t>
+          <t>Jl. Kayu Manis Barat No. 15 RT 019/004 Kayu Manis</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>Cimanggis</t>
+          <t>Kayu Manis</t>
         </is>
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>Cimanggis</t>
+          <t>Matraman</t>
         </is>
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>Depok</t>
+          <t>Jakarta Timur</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>Jawa Barat</t>
+          <t>DKI Jakarta</t>
         </is>
       </c>
       <c r="J151" t="inlineStr">
         <is>
-          <t>12.7 KM</t>
+          <t>12 KM</t>
         </is>
       </c>
       <c r="K151" t="inlineStr">
@@ -9123,35 +9123,35 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Imam Santoso</t>
+          <t>Rahayu Ningsih</t>
         </is>
       </c>
       <c r="C152" t="n">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>Laki - Laki</t>
+          <t>Perempuan</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>Jl. Cilandak No. 64, RT.005/RW.003</t>
+          <t>Jl. Garuda VII Pulo Gebang Permai No. 5 RT 002/003</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>Guntur</t>
+          <t>Pulo Gebang</t>
         </is>
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>Setiabudi</t>
+          <t>Cakung</t>
         </is>
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>Jakarta Selatan</t>
+          <t>Jakarta Timur</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
@@ -9161,7 +9161,7 @@
       </c>
       <c r="J152" t="inlineStr">
         <is>
-          <t>7.8 KM</t>
+          <t>11 KM</t>
         </is>
       </c>
       <c r="K152" t="inlineStr">
@@ -9171,7 +9171,7 @@
       </c>
       <c r="L152" t="inlineStr">
         <is>
-          <t>Hadir</t>
+          <t>Tidak Hadir</t>
         </is>
       </c>
     </row>
@@ -9181,30 +9181,30 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Ridwan Tambunan</t>
+          <t>Suhartini</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>Laki - Laki</t>
+          <t>Perempuan</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>Jl. Ciracas No. 118 RT 06 RW 05</t>
+          <t>Jl. Dewi Sartika No. 8 RT 003/005 Cililitan</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>Lubang Buaya</t>
+          <t>Cililitan</t>
         </is>
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>Cipayung</t>
+          <t>Kramat Jati</t>
         </is>
       </c>
       <c r="H153" t="inlineStr">
@@ -9219,7 +9219,7 @@
       </c>
       <c r="J153" t="inlineStr">
         <is>
-          <t>6.4 KM</t>
+          <t>2 KM</t>
         </is>
       </c>
       <c r="K153" t="inlineStr">

</xml_diff>

<commit_message>
Anonymize dataset + add setup.md, 00_anonymize.py, backup, retrain model
</commit_message>
<xml_diff>
--- a/data/raw/event1_raw.xlsx
+++ b/data/raw/event1_raw.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Peserta" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,24 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -57,17 +46,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -435,92 +415,100 @@
   </sheetPr>
   <dimension ref="A1:L153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="6" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-  </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1">
+      <c r="A1" t="inlineStr">
         <is>
           <t>PESERTA PELATIHAN MAKANAN VIRAL SUSHI &amp; ONIGIRI</t>
         </is>
       </c>
-    </row>
-    <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="B1" t="inlineStr"/>
+      <c r="C1" t="inlineStr"/>
+      <c r="D1" t="inlineStr"/>
+      <c r="E1" t="inlineStr"/>
+      <c r="F1" t="inlineStr"/>
+      <c r="G1" t="inlineStr"/>
+      <c r="H1" t="inlineStr"/>
+      <c r="I1" t="inlineStr"/>
+      <c r="J1" t="inlineStr"/>
+      <c r="K1" t="inlineStr"/>
+      <c r="L1" t="inlineStr"/>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
         <is>
           <t>MINGGU, 09 NOVEMBER 2025</t>
         </is>
       </c>
-    </row>
-    <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>ID ANGGOTA</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Usia</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Jenis Kelamin</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Alamat tempat tinggal</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Desa/Kelurahan</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Kecamatan</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>Kabupaten/Kota</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>Provinsi</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>Jarak</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>Status Pendaftaran</t>
         </is>
       </c>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>Status Kehadiran</t>
         </is>
@@ -532,7 +520,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Rosmiyanti</t>
+          <t>P149</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -590,7 +578,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Agusnawati</t>
+          <t>P005</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -648,7 +636,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Dra.Endaruna</t>
+          <t>P046</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -707,7 +695,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Soraya safitri</t>
+          <t>P165</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -765,7 +753,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Asep Sudjana</t>
+          <t>P017</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -824,7 +812,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Chairunnisyah Nst</t>
+          <t>P028</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -882,7 +870,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Shanty Puspa oktavianty</t>
+          <t>P154</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -940,7 +928,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Sri hartaty</t>
+          <t>P166</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -998,7 +986,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Ambar Kriswijayanti</t>
+          <t>P011</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1056,7 +1044,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Jl kp Pulo nrt 6 RW 5 pinang Ranti</t>
+          <t>P139</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -1114,7 +1102,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Elok Lisawaty</t>
+          <t>P054</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -1172,7 +1160,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Siti Rochanah</t>
+          <t>P159</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -1230,7 +1218,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Robiatul adawiyah</t>
+          <t>P143</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -1288,7 +1276,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Anna luciana</t>
+          <t>P016</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -1346,7 +1334,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>SUZAN.TRI WAHYUNI</t>
+          <t>P186</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -1404,7 +1392,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Desi Rofiqo Hermawati</t>
+          <t>P040</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -1462,7 +1450,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Sri Oktaviyani</t>
+          <t>P167</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -1520,7 +1508,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Sitti fauziawati</t>
+          <t>P161</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -1578,7 +1566,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Winarsih</t>
+          <t>P207</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -1636,7 +1624,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Ekka JuniHarni Putri</t>
+          <t>P052</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -1694,7 +1682,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Siti chairiyah</t>
+          <t>P156</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -1752,7 +1740,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>INDAH PERMATA SARI</t>
+          <t>P079</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -1810,7 +1798,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>DWI JOKO PURWONO</t>
+          <t>P047</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -1868,7 +1856,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Derisma wahyuni</t>
+          <t>P039</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -1926,7 +1914,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>RAHMAT FAUZI</t>
+          <t>P136</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -1984,7 +1972,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Endang Budiyanti</t>
+          <t>P056</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -2042,7 +2030,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Nunik Damiasih</t>
+          <t>P125</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -2100,7 +2088,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Kurnia Agustina</t>
+          <t>P096</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -2158,7 +2146,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Indah Widyawati</t>
+          <t>P080</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -2216,7 +2204,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Nindra diyanti</t>
+          <t>P123</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -2275,7 +2263,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Puryat i</t>
+          <t>P135</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -2333,7 +2321,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Najwa aulia rahman</t>
+          <t>P116</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -2391,7 +2379,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>SURATMI</t>
+          <t>P183</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -2450,7 +2438,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>zelfi zafira</t>
+          <t>P220</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -2508,7 +2496,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Susanti</t>
+          <t>P184</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -2567,7 +2555,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Ineke Fransiska fortunata</t>
+          <t>P081</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -2625,7 +2613,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Warti Ruliana</t>
+          <t>P206</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -2683,7 +2671,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Juwita Laraswaty</t>
+          <t>P086</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -2741,7 +2729,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Asrifah</t>
+          <t>P018</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -2800,7 +2788,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Soleha.n</t>
+          <t>P164</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -2858,7 +2846,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Sumiyati</t>
+          <t>P176</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -2916,7 +2904,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Rini pujiastuti</t>
+          <t>P142</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -2974,7 +2962,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Sadiyah</t>
+          <t>P152</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -3032,7 +3020,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Maina Karnita</t>
+          <t>P103</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -3090,7 +3078,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Budi Ristanto</t>
+          <t>P024</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -3148,7 +3136,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Vera Anggraeni</t>
+          <t>P204</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -3206,7 +3194,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Suswati</t>
+          <t>P185</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -3264,7 +3252,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Hety meilati</t>
+          <t>P076</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -3322,7 +3310,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>ENDAH NURPITA</t>
+          <t>P055</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -3381,7 +3369,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>OON KARWATI</t>
+          <t>P130</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -3439,7 +3427,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>SITI NURHAYATI</t>
+          <t>P158</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -3497,7 +3485,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>SRI WAHYUNINGSIH</t>
+          <t>P168</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -3555,7 +3543,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Berti</t>
+          <t>P022</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -3613,7 +3601,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Eti Nurbaiti</t>
+          <t>P061</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -3671,7 +3659,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Malinda</t>
+          <t>P105</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -3729,7 +3717,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>DIAH MuZTINNINGRUM</t>
+          <t>P044</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -3787,7 +3775,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>WULAN KINASIH</t>
+          <t>P209</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -3845,7 +3833,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Julaeha Rahayu</t>
+          <t>P085</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -3903,7 +3891,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Dwi Murniasih</t>
+          <t>P048</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -3961,7 +3949,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Ahmad subana</t>
+          <t>P006</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -4019,7 +4007,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Sumiyati</t>
+          <t>P108</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -4077,7 +4065,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Afriyati Utami</t>
+          <t>P003</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -4135,7 +4123,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Priyanti Lestari</t>
+          <t>P132</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -4193,7 +4181,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Sukiyem</t>
+          <t>P171</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -4251,7 +4239,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Titin Abdullah</t>
+          <t>P192</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -4309,7 +4297,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Dahlia Sukowati</t>
+          <t>P034</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -4367,7 +4355,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Neneng</t>
+          <t>P122</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -4425,7 +4413,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Jubaedah Indah</t>
+          <t>P083</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -4483,7 +4471,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Titin Mulyati</t>
+          <t>P193</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -4541,7 +4529,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Uyi Nanda Prasaja</t>
+          <t>P200</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -4599,7 +4587,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>USMUNAH</t>
+          <t>P199</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -4657,7 +4645,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Nur Darsitah</t>
+          <t>P126</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -4715,7 +4703,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Muchlid Noor</t>
+          <t>P109</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -4773,7 +4761,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Siti Mardiana</t>
+          <t>P157</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -4831,7 +4819,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Yolanda Hutapea</t>
+          <t>P214</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -4889,7 +4877,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Syarifah</t>
+          <t>P187</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -4947,7 +4935,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Indah Juniar</t>
+          <t>P078</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -5005,7 +4993,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Dewi Julianti</t>
+          <t>P041</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -5063,7 +5051,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>YUYUN</t>
+          <t>P216</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -5121,7 +5109,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Citra Dewi Sofian</t>
+          <t>P033</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -5179,7 +5167,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Karmini Anubhawa</t>
+          <t>P089</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -5237,7 +5225,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Rina Marlina</t>
+          <t>P138</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -5295,7 +5283,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Erna wulandari</t>
+          <t>P059</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -5353,7 +5341,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Tuti Herawati</t>
+          <t>P197</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -5411,7 +5399,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Dewi Kartika Sari</t>
+          <t>P042</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -5469,7 +5457,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Ani Lestari</t>
+          <t>P013</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -5527,7 +5515,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Eti Sunarsih</t>
+          <t>P062</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -5585,7 +5573,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Nanik Puji Astuti</t>
+          <t>P118</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -5643,7 +5631,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Tri Susilowati</t>
+          <t>P196</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -5701,7 +5689,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Tatik Kusumawati</t>
+          <t>P189</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -5759,7 +5747,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Lilis</t>
+          <t>P101</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -5817,7 +5805,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Hartingsih</t>
+          <t>P070</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -5875,7 +5863,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Sulastri Mulyani</t>
+          <t>P172</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -5933,7 +5921,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sunarto </t>
+          <t>P179</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -5991,7 +5979,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Luluk Maesaroh</t>
+          <t>P102</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -6049,7 +6037,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Titin Sumarni</t>
+          <t>P194</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -6107,7 +6095,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Wiwin Oktaviani</t>
+          <t>P208</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -6165,7 +6153,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Dian Kusuma Ningrum</t>
+          <t>P045</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -6223,7 +6211,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Yanti Nurlela</t>
+          <t>P212</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -6281,7 +6269,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Rosita Handayaningsih</t>
+          <t>P148</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -6339,7 +6327,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Mardiana</t>
+          <t>P032</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -6397,7 +6385,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Aisyah Putri</t>
+          <t>P007</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -6455,7 +6443,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Supiah</t>
+          <t>P180</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -6513,7 +6501,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Nuraini</t>
+          <t>P067</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -6571,7 +6559,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Agus Salim</t>
+          <t>P004</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -6629,7 +6617,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Umi Salamah</t>
+          <t>P198</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -6687,7 +6675,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Nurjanah</t>
+          <t>P019</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -6745,7 +6733,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Sunarti</t>
+          <t>P178</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -6803,7 +6791,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Fatmawati</t>
+          <t>P068</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -6861,7 +6849,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Maisyaroh</t>
+          <t>P104</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -6919,7 +6907,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Murniati</t>
+          <t>P111</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -6977,7 +6965,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Komariah</t>
+          <t>P112</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -7035,7 +7023,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Hayati</t>
+          <t>P074</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -7093,7 +7081,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Wahyu Santoso</t>
+          <t>P205</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -7151,7 +7139,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Eka Fitriani</t>
+          <t>P049</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -7209,7 +7197,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Aminah</t>
+          <t>P012</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -7267,7 +7255,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Supriyati</t>
+          <t>P182</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -7325,7 +7313,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Hindun</t>
+          <t>P077</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -7383,7 +7371,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Wulandari</t>
+          <t>P211</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -7441,7 +7429,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Dewi Lestari</t>
+          <t>P043</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -7499,7 +7487,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Endang Susanti</t>
+          <t>P115</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -7557,7 +7545,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Nurhayati</t>
+          <t>P091</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -7615,7 +7603,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Erni Rahayu</t>
+          <t>P060</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -7673,7 +7661,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Wati Susanti</t>
+          <t>P008</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -7731,7 +7719,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Siti Rohani</t>
+          <t>P160</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -7789,7 +7777,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Wahyuni</t>
+          <t>P219</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -7847,7 +7835,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Srimulyani</t>
+          <t>P169</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -7905,7 +7893,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Teti Haryati</t>
+          <t>P190</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -7963,7 +7951,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Suryani</t>
+          <t>P120</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -8021,7 +8009,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Rubiyah</t>
+          <t>P150</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -8079,7 +8067,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Adi Prasetyo</t>
+          <t>P002</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -8137,7 +8125,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Rosdiana</t>
+          <t>P147</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -8195,7 +8183,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Sumiarsih</t>
+          <t>P174</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -8253,7 +8241,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Eko Purnomo</t>
+          <t>P053</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -8311,7 +8299,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Titin Suprihatin</t>
+          <t>P195</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -8369,7 +8357,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Septiani</t>
+          <t>P218</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -8427,7 +8415,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Hartini</t>
+          <t>P072</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -8485,7 +8473,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Pariyem</t>
+          <t>P131</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -8543,7 +8531,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Salmah</t>
+          <t>P153</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -8601,7 +8589,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Novia Anggraeni</t>
+          <t>P124</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -8659,7 +8647,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>Karmiati</t>
+          <t>P088</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -8717,7 +8705,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Lela Wati</t>
+          <t>P100</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -8775,7 +8763,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>Yayah Sumiyah</t>
+          <t>P213</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -8833,7 +8821,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Mariana Sari</t>
+          <t>P202</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -8891,7 +8879,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Cicih Suryani</t>
+          <t>P031</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -8949,7 +8937,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Rini Handayani</t>
+          <t>P140</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -9007,7 +8995,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Budi Hartono</t>
+          <t>P023</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -9065,7 +9053,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>Hermanto</t>
+          <t>P075</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -9123,7 +9111,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Rahayu Ningsih</t>
+          <t>P030</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -9181,7 +9169,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Suhartini</t>
+          <t>P009</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -9234,10 +9222,6 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:L2"/>
-    <mergeCell ref="A1:L1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>